<commit_message>
Update Other Comprehensive Income Feature
</commit_message>
<xml_diff>
--- a/data/summarized fitur kpmm - KBMI 4.xlsx
+++ b/data/summarized fitur kpmm - KBMI 4.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K89"/>
+  <dimension ref="A1:L89"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,6 +488,11 @@
           <t>modal_terhadap_kredit_bersih</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>other_comprehensive_income_to_equity</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="n">
@@ -529,6 +534,7 @@
       </c>
       <c r="J2" t="inlineStr"/>
       <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -570,6 +576,7 @@
       </c>
       <c r="J3" t="inlineStr"/>
       <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="n">
@@ -611,6 +618,7 @@
       </c>
       <c r="J4" t="inlineStr"/>
       <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -652,6 +660,7 @@
       </c>
       <c r="J5" t="inlineStr"/>
       <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -697,6 +706,9 @@
       <c r="K6" t="n">
         <v>0.2797359135425686</v>
       </c>
+      <c r="L6" t="n">
+        <v>0.06796463630589007</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -742,6 +754,9 @@
       <c r="K7" t="n">
         <v>0.2348764578158021</v>
       </c>
+      <c r="L7" t="n">
+        <v>0.160743318935699</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -787,6 +802,9 @@
       <c r="K8" t="n">
         <v>0.2209259826972046</v>
       </c>
+      <c r="L8" t="n">
+        <v>0.1270230357512929</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -832,6 +850,9 @@
       <c r="K9" t="n">
         <v>0.2275362634845475</v>
       </c>
+      <c r="L9" t="n">
+        <v>0.08637087421332146</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
@@ -873,6 +894,7 @@
       </c>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
+      <c r="L10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -914,6 +936,7 @@
       </c>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
+      <c r="L11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -955,6 +978,7 @@
       </c>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
+      <c r="L12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
@@ -996,6 +1020,7 @@
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
+      <c r="L13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1037,6 +1062,7 @@
       </c>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1078,6 +1104,7 @@
       </c>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1119,6 +1146,7 @@
       </c>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -1160,6 +1188,7 @@
       </c>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1205,6 +1234,9 @@
       <c r="K18" t="n">
         <v>0.2969280653106242</v>
       </c>
+      <c r="L18" t="n">
+        <v>0.08339051527641031</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
@@ -1250,6 +1282,9 @@
       <c r="K19" t="n">
         <v>0.2226456915884258</v>
       </c>
+      <c r="L19" t="n">
+        <v>0.1902418966912749</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1295,6 +1330,9 @@
       <c r="K20" t="n">
         <v>0.189592638930083</v>
       </c>
+      <c r="L20" t="n">
+        <v>0.1443376998689689</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1340,6 +1378,9 @@
       <c r="K21" t="n">
         <v>0.2085579151625621</v>
       </c>
+      <c r="L21" t="n">
+        <v>0.1108474205787282</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -1385,6 +1426,9 @@
       <c r="K22" t="n">
         <v>0.305619590777283</v>
       </c>
+      <c r="L22" t="n">
+        <v>0.09290745137429467</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -1430,6 +1474,9 @@
       <c r="K23" t="n">
         <v>0.2213571090860221</v>
       </c>
+      <c r="L23" t="n">
+        <v>0.19501058044562</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -1475,6 +1522,9 @@
       <c r="K24" t="n">
         <v>0.1901481098393105</v>
       </c>
+      <c r="L24" t="n">
+        <v>0.1631424359520917</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
@@ -1520,6 +1570,9 @@
       <c r="K25" t="n">
         <v>0.2140615295973768</v>
       </c>
+      <c r="L25" t="n">
+        <v>0.1141448163307525</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -1565,6 +1618,9 @@
       <c r="K26" t="n">
         <v>0.2942458223686331</v>
       </c>
+      <c r="L26" t="n">
+        <v>0.08308610002847283</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
@@ -1610,6 +1666,9 @@
       <c r="K27" t="n">
         <v>0.2040866668241209</v>
       </c>
+      <c r="L27" t="n">
+        <v>0.188397518399739</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -1655,6 +1714,9 @@
       <c r="K28" t="n">
         <v>0.1896129664155844</v>
       </c>
+      <c r="L28" t="n">
+        <v>0.1448481104192894</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
@@ -1700,6 +1762,9 @@
       <c r="K29" t="n">
         <v>0.2036247519459581</v>
       </c>
+      <c r="L29" t="n">
+        <v>0.1025223702852764</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -1745,6 +1810,9 @@
       <c r="K30" t="n">
         <v>0.3081068766957478</v>
       </c>
+      <c r="L30" t="n">
+        <v>0.08603281206994173</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -1790,6 +1858,9 @@
       <c r="K31" t="n">
         <v>0.2065346572907454</v>
       </c>
+      <c r="L31" t="n">
+        <v>0.1817376553455033</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -1835,6 +1906,9 @@
       <c r="K32" t="n">
         <v>0.1899101961976699</v>
       </c>
+      <c r="L32" t="n">
+        <v>0.1437018266814244</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -1880,6 +1954,9 @@
       <c r="K33" t="n">
         <v>0.2079733482723117</v>
       </c>
+      <c r="L33" t="n">
+        <v>0.1038057173719232</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -1925,6 +2002,9 @@
       <c r="K34" t="n">
         <v>0.3165044067837977</v>
       </c>
+      <c r="L34" t="n">
+        <v>0.08249555595374546</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -1970,6 +2050,9 @@
       <c r="K35" t="n">
         <v>0.2136903060052048</v>
       </c>
+      <c r="L35" t="n">
+        <v>0.1772494510444146</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -2015,6 +2098,9 @@
       <c r="K36" t="n">
         <v>0.194982905080584</v>
       </c>
+      <c r="L36" t="n">
+        <v>0.1410302832007156</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -2060,6 +2146,9 @@
       <c r="K37" t="n">
         <v>0.2605600115771484</v>
       </c>
+      <c r="L37" t="n">
+        <v>0.06784953501243152</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -2105,6 +2194,9 @@
       <c r="K38" t="n">
         <v>0.3082915945370628</v>
       </c>
+      <c r="L38" t="n">
+        <v>0.07950253103100267</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -2150,6 +2242,9 @@
       <c r="K39" t="n">
         <v>0.2160816513161762</v>
       </c>
+      <c r="L39" t="n">
+        <v>0.1658420685251212</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -2195,6 +2290,9 @@
       <c r="K40" t="n">
         <v>0.1966213508831904</v>
       </c>
+      <c r="L40" t="n">
+        <v>0.1445904163557597</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -2240,6 +2338,9 @@
       <c r="K41" t="n">
         <v>0.269485081193689</v>
       </c>
+      <c r="L41" t="n">
+        <v>0.06726710247294171</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -2285,6 +2386,9 @@
       <c r="K42" t="n">
         <v>0.3464095375013367</v>
       </c>
+      <c r="L42" t="n">
+        <v>0.07625198104489955</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
@@ -2330,6 +2434,9 @@
       <c r="K43" t="n">
         <v>0.2727110956880541</v>
       </c>
+      <c r="L43" t="n">
+        <v>0.1940212157383863</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -2375,6 +2482,9 @@
       <c r="K44" t="n">
         <v>0.240935707962027</v>
       </c>
+      <c r="L44" t="n">
+        <v>0.1269794612264487</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -2420,6 +2530,9 @@
       <c r="K45" t="n">
         <v>0.2869840846865587</v>
       </c>
+      <c r="L45" t="n">
+        <v>0.0746079445978037</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -2465,6 +2578,9 @@
       <c r="K46" t="n">
         <v>0.3485561259835385</v>
       </c>
+      <c r="L46" t="n">
+        <v>0.06850952520990221</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -2510,6 +2626,9 @@
       <c r="K47" t="n">
         <v>0.2729211016585265</v>
       </c>
+      <c r="L47" t="n">
+        <v>0.1900908270490136</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -2555,6 +2674,9 @@
       <c r="K48" t="n">
         <v>0.2269934742957803</v>
       </c>
+      <c r="L48" t="n">
+        <v>0.1265004909022094</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
@@ -2600,6 +2722,9 @@
       <c r="K49" t="n">
         <v>0.2913061747690214</v>
       </c>
+      <c r="L49" t="n">
+        <v>0.07211784610299479</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -2645,6 +2770,9 @@
       <c r="K50" t="n">
         <v>0.3624020608149472</v>
       </c>
+      <c r="L50" t="n">
+        <v>0.06045961547614706</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -2690,6 +2818,9 @@
       <c r="K51" t="n">
         <v>0.2828200296229214</v>
       </c>
+      <c r="L51" t="n">
+        <v>0.17829292985725</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -2735,6 +2866,9 @@
       <c r="K52" t="n">
         <v>0.2312586367322242</v>
       </c>
+      <c r="L52" t="n">
+        <v>0.12287448335342</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -2780,6 +2914,9 @@
       <c r="K53" t="n">
         <v>0.3051904514105914</v>
       </c>
+      <c r="L53" t="n">
+        <v>0.06889670893430648</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
@@ -2825,6 +2962,9 @@
       <c r="K54" t="n">
         <v>0.3558940069958999</v>
       </c>
+      <c r="L54" t="n">
+        <v>0.05843625112722368</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
@@ -2870,6 +3010,9 @@
       <c r="K55" t="n">
         <v>0.2953964235771921</v>
       </c>
+      <c r="L55" t="n">
+        <v>0.164793293647807</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
@@ -2915,6 +3058,9 @@
       <c r="K56" t="n">
         <v>0.2339545810995853</v>
       </c>
+      <c r="L56" t="n">
+        <v>0.1170831922209005</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -2960,6 +3106,9 @@
       <c r="K57" t="n">
         <v>0.3009992186544527</v>
       </c>
+      <c r="L57" t="n">
+        <v>0.06851686233243989</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -3005,6 +3154,9 @@
       <c r="K58" t="n">
         <v>0.3324221071779174</v>
       </c>
+      <c r="L58" t="n">
+        <v>0.06089360037268897</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -3050,6 +3202,9 @@
       <c r="K59" t="n">
         <v>0.2758364947360882</v>
       </c>
+      <c r="L59" t="n">
+        <v>0.1772774077905052</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -3095,6 +3250,9 @@
       <c r="K60" t="n">
         <v>0.2305086375203145</v>
       </c>
+      <c r="L60" t="n">
+        <v>0.1129998637296999</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -3140,6 +3298,9 @@
       <c r="K61" t="n">
         <v>0.2724958192465747</v>
       </c>
+      <c r="L61" t="n">
+        <v>0.07444250148500142</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -3185,6 +3346,9 @@
       <c r="K62" t="n">
         <v>0.341922369009644</v>
       </c>
+      <c r="L62" t="n">
+        <v>0.05922524991279196</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -3230,6 +3394,9 @@
       <c r="K63" t="n">
         <v>0.2754349969659436</v>
       </c>
+      <c r="L63" t="n">
+        <v>0.1674388418464859</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -3275,6 +3442,9 @@
       <c r="K64" t="n">
         <v>0.2318944563064989</v>
       </c>
+      <c r="L64" t="n">
+        <v>0.1145279976453218</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -3320,6 +3490,9 @@
       <c r="K65" t="n">
         <v>0.277569223762868</v>
       </c>
+      <c r="L65" t="n">
+        <v>0.07065807755196744</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -3365,6 +3538,9 @@
       <c r="K66" t="n">
         <v>0.3491304981466885</v>
       </c>
+      <c r="L66" t="n">
+        <v>0.05591537623813841</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
@@ -3410,6 +3586,9 @@
       <c r="K67" t="n">
         <v>0.2852568194446819</v>
       </c>
+      <c r="L67" t="n">
+        <v>0.1607560911367578</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
@@ -3455,6 +3634,9 @@
       <c r="K68" t="n">
         <v>0.2185149808410252</v>
       </c>
+      <c r="L68" t="n">
+        <v>0.1131488243456331</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -3500,6 +3682,9 @@
       <c r="K69" t="n">
         <v>0.2813933952534939</v>
       </c>
+      <c r="L69" t="n">
+        <v>0.06818586821917513</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
@@ -3545,6 +3730,9 @@
       <c r="K70" t="n">
         <v>0.3387951074270932</v>
       </c>
+      <c r="L70" t="n">
+        <v>0.05103587967748134</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
@@ -3590,6 +3778,9 @@
       <c r="K71" t="n">
         <v>0.2753915974522796</v>
       </c>
+      <c r="L71" t="n">
+        <v>0.1476133435169871</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
@@ -3635,6 +3826,9 @@
       <c r="K72" t="n">
         <v>0.2154985954296849</v>
       </c>
+      <c r="L72" t="n">
+        <v>0.1143864122723514</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
@@ -3680,6 +3874,9 @@
       <c r="K73" t="n">
         <v>0.2731723416669541</v>
       </c>
+      <c r="L73" t="n">
+        <v>0.06736333058586796</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
@@ -3725,6 +3922,9 @@
       <c r="K74" t="n">
         <v>0.2602954251096185</v>
       </c>
+      <c r="L74" t="n">
+        <v>0.05397168161951788</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -3770,6 +3970,9 @@
       <c r="K75" t="n">
         <v>0.1765265400429891</v>
       </c>
+      <c r="L75" t="n">
+        <v>0.1608613511713409</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
@@ -3815,6 +4018,9 @@
       <c r="K76" t="n">
         <v>0.1823490389158245</v>
       </c>
+      <c r="L76" t="n">
+        <v>0.1092185888382411</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -3860,6 +4066,9 @@
       <c r="K77" t="n">
         <v>0.1996045386445293</v>
       </c>
+      <c r="L77" t="n">
+        <v>0.07190358217245034</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
@@ -3905,6 +4114,9 @@
       <c r="K78" t="n">
         <v>0.273419054563257</v>
       </c>
+      <c r="L78" t="n">
+        <v>0.04868721380627796</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -3950,6 +4162,9 @@
       <c r="K79" t="n">
         <v>0.1762803218354767</v>
       </c>
+      <c r="L79" t="n">
+        <v>0.1504646068793182</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
@@ -3995,6 +4210,9 @@
       <c r="K80" t="n">
         <v>0.1799393639382263</v>
       </c>
+      <c r="L80" t="n">
+        <v>0.1059027167869239</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
@@ -4040,6 +4258,9 @@
       <c r="K81" t="n">
         <v>0.2073837624239262</v>
       </c>
+      <c r="L81" t="n">
+        <v>0.06796738779873704</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -4085,6 +4306,9 @@
       <c r="K82" t="n">
         <v>0.2829393989410953</v>
       </c>
+      <c r="L82" t="n">
+        <v>0.04904944114986653</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -4130,6 +4354,9 @@
       <c r="K83" t="n">
         <v>0.1838951011059687</v>
       </c>
+      <c r="L83" t="n">
+        <v>0.1423512806881353</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -4175,6 +4402,9 @@
       <c r="K84" t="n">
         <v>0.189826201883504</v>
       </c>
+      <c r="L84" t="n">
+        <v>0.1015396911195705</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
@@ -4220,6 +4450,9 @@
       <c r="K85" t="n">
         <v>0.2187709537446556</v>
       </c>
+      <c r="L85" t="n">
+        <v>0.06478323733358667</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="n">
@@ -4265,6 +4498,9 @@
       <c r="K86" t="n">
         <v>0.277933993644305</v>
       </c>
+      <c r="L86" t="n">
+        <v>0.04465238529659792</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -4310,6 +4546,9 @@
       <c r="K87" t="n">
         <v>0.1808960914304709</v>
       </c>
+      <c r="L87" t="n">
+        <v>0.1344340699219137</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="n">
@@ -4355,6 +4594,9 @@
       <c r="K88" t="n">
         <v>0.1833498593896899</v>
       </c>
+      <c r="L88" t="n">
+        <v>0.1052911801499009</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="n">
@@ -4399,6 +4641,9 @@
       </c>
       <c r="K89" t="n">
         <v>0.210843251123958</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0.06629227233985083</v>
       </c>
     </row>
   </sheetData>

</xml_diff>